<commit_message>
Updated NABOS Run Details
Updated NABOS Run -- compared to June 19 output. Includes Filter & CellTM, need to produce final file.
</commit_message>
<xml_diff>
--- a/output/nabos_01_01avg.xlsx
+++ b/output/nabos_01_01avg.xlsx
@@ -541,10 +541,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2.969</v>
+        <v>2.96</v>
       </c>
       <c r="B2" t="n">
-        <v>73.77058</v>
+        <v>73.77059</v>
       </c>
       <c r="C2" t="n">
         <v>167.71341</v>
@@ -553,64 +553,64 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.6549</v>
+        <v>-0.6566</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.6555</v>
+        <v>-0.6575</v>
       </c>
       <c r="G2" t="n">
-        <v>22.273449</v>
+        <v>22.274264</v>
       </c>
       <c r="H2" t="n">
-        <v>22.275594</v>
+        <v>22.276062</v>
       </c>
       <c r="I2" t="n">
-        <v>26.724</v>
+        <v>26.7266</v>
       </c>
       <c r="J2" t="n">
-        <v>26.7274</v>
+        <v>26.7297</v>
       </c>
       <c r="K2" t="n">
-        <v>371.01</v>
+        <v>371.087</v>
       </c>
       <c r="L2" t="n">
-        <v>362.495</v>
+        <v>362.564</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0915</v>
+        <v>0.0894</v>
       </c>
       <c r="N2" t="n">
-        <v>4.5683</v>
+        <v>4.5697</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1009</v>
+        <v>0.1012</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1009</v>
+        <v>0.1012</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1043</v>
+        <v>0.1031</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0287</v>
+        <v>0.0286</v>
       </c>
       <c r="S2" t="n">
-        <v>6371</v>
+        <v>6374</v>
       </c>
       <c r="T2" t="n">
-        <v>4.4239</v>
+        <v>4.426</v>
       </c>
       <c r="U2" t="n">
-        <v>26.22</v>
+        <v>25.93</v>
       </c>
       <c r="V2" t="n">
-        <v>2.6027</v>
+        <v>2.603</v>
       </c>
       <c r="W2" t="n">
-        <v>2.261</v>
+        <v>2.2612</v>
       </c>
       <c r="X2" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -633,7 +633,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3.959</v>
+        <v>3.958</v>
       </c>
       <c r="B3" t="n">
         <v>73.77057</v>
@@ -645,34 +645,34 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.6805</v>
+        <v>-0.6811</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.6789</v>
+        <v>-0.6799</v>
       </c>
       <c r="G3" t="n">
-        <v>22.27592</v>
+        <v>22.274977</v>
       </c>
       <c r="H3" t="n">
-        <v>22.275171</v>
+        <v>22.274888</v>
       </c>
       <c r="I3" t="n">
-        <v>26.7495</v>
+        <v>26.7494</v>
       </c>
       <c r="J3" t="n">
-        <v>26.7471</v>
+        <v>26.7481</v>
       </c>
       <c r="K3" t="n">
-        <v>371.42</v>
+        <v>371.418</v>
       </c>
       <c r="L3" t="n">
-        <v>362.943</v>
+        <v>363.021</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1025</v>
+        <v>0.1044</v>
       </c>
       <c r="N3" t="n">
-        <v>4.5701</v>
+        <v>4.5706</v>
       </c>
       <c r="O3" t="n">
         <v>0.1028</v>
@@ -681,28 +681,28 @@
         <v>0.1028</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.1028</v>
+        <v>0.1023</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0291</v>
+        <v>0.0292</v>
       </c>
       <c r="S3" t="n">
-        <v>6468</v>
+        <v>6475</v>
       </c>
       <c r="T3" t="n">
-        <v>4.4913</v>
+        <v>4.496</v>
       </c>
       <c r="U3" t="n">
-        <v>27.88</v>
+        <v>27.9</v>
       </c>
       <c r="V3" t="n">
-        <v>2.6035</v>
+        <v>2.6034</v>
       </c>
       <c r="W3" t="n">
-        <v>2.2619</v>
+        <v>2.2623</v>
       </c>
       <c r="X3" t="n">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="Y3" t="n">
         <v>0</v>
@@ -725,7 +725,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4.948</v>
+        <v>4.95</v>
       </c>
       <c r="B4" t="n">
         <v>73.77056</v>
@@ -737,34 +737,34 @@
         <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.6861</v>
+        <v>-0.6863</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.6857</v>
+        <v>-0.6859</v>
       </c>
       <c r="G4" t="n">
-        <v>22.279733</v>
+        <v>22.279389</v>
       </c>
       <c r="H4" t="n">
-        <v>22.277331</v>
+        <v>22.277162</v>
       </c>
       <c r="I4" t="n">
-        <v>26.759</v>
+        <v>26.7591</v>
       </c>
       <c r="J4" t="n">
-        <v>26.7555</v>
+        <v>26.7558</v>
       </c>
       <c r="K4" t="n">
-        <v>371.669</v>
+        <v>371.659</v>
       </c>
       <c r="L4" t="n">
-        <v>362.909</v>
+        <v>362.932</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1174</v>
+        <v>0.1172</v>
       </c>
       <c r="N4" t="n">
-        <v>4.5748</v>
+        <v>4.5749</v>
       </c>
       <c r="O4" t="n">
         <v>0.1014</v>
@@ -773,28 +773,28 @@
         <v>0.1014</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0987</v>
+        <v>0.0985</v>
       </c>
       <c r="R4" t="n">
         <v>0.0297</v>
       </c>
       <c r="S4" t="n">
-        <v>6563</v>
+        <v>6565</v>
       </c>
       <c r="T4" t="n">
-        <v>4.5566</v>
+        <v>4.558</v>
       </c>
       <c r="U4" t="n">
-        <v>26.36</v>
+        <v>26.25</v>
       </c>
       <c r="V4" t="n">
         <v>2.6044</v>
       </c>
       <c r="W4" t="n">
-        <v>2.2613</v>
+        <v>2.2614</v>
       </c>
       <c r="X4" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="Y4" t="n">
         <v>0</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5.938</v>
+        <v>5.936</v>
       </c>
       <c r="B5" t="n">
         <v>73.77056</v>
@@ -829,64 +829,64 @@
         <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.6846</v>
+        <v>-0.685</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.6842</v>
+        <v>-0.6849</v>
       </c>
       <c r="G5" t="n">
-        <v>22.277575</v>
+        <v>22.2777</v>
       </c>
       <c r="H5" t="n">
-        <v>22.276403</v>
+        <v>22.276677</v>
       </c>
       <c r="I5" t="n">
-        <v>26.7542</v>
+        <v>26.755</v>
       </c>
       <c r="J5" t="n">
-        <v>26.7524</v>
+        <v>26.7536</v>
       </c>
       <c r="K5" t="n">
-        <v>371.461</v>
+        <v>371.548</v>
       </c>
       <c r="L5" t="n">
-        <v>362.849</v>
+        <v>362.481</v>
       </c>
       <c r="M5" t="n">
-        <v>0.111</v>
+        <v>0.1166</v>
       </c>
       <c r="N5" t="n">
-        <v>4.5729</v>
+        <v>4.5723</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1026</v>
+        <v>0.1019</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1026</v>
+        <v>0.1019</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1002</v>
+        <v>0.1008</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0294</v>
+        <v>0.0297</v>
       </c>
       <c r="S5" t="n">
-        <v>6653</v>
+        <v>6659</v>
       </c>
       <c r="T5" t="n">
-        <v>4.6198</v>
+        <v>4.6236</v>
       </c>
       <c r="U5" t="n">
-        <v>25.91</v>
+        <v>25.29</v>
       </c>
       <c r="V5" t="n">
-        <v>2.603</v>
+        <v>2.6035</v>
       </c>
       <c r="W5" t="n">
-        <v>2.2608</v>
+        <v>2.259</v>
       </c>
       <c r="X5" t="n">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="Y5" t="n">
         <v>0</v>
@@ -909,7 +909,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6.928</v>
+        <v>6.927</v>
       </c>
       <c r="B6" t="n">
         <v>73.77056</v>
@@ -921,64 +921,64 @@
         <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.668</v>
+        <v>-0.6694</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.6697</v>
+        <v>-0.6703</v>
       </c>
       <c r="G6" t="n">
-        <v>22.284377</v>
+        <v>22.285989</v>
       </c>
       <c r="H6" t="n">
-        <v>22.281008</v>
+        <v>22.281983</v>
       </c>
       <c r="I6" t="n">
-        <v>26.748</v>
+        <v>26.7511</v>
       </c>
       <c r="J6" t="n">
-        <v>26.7451</v>
+        <v>26.7466</v>
       </c>
       <c r="K6" t="n">
-        <v>371.359</v>
+        <v>371.378</v>
       </c>
       <c r="L6" t="n">
-        <v>362.736</v>
+        <v>362.684</v>
       </c>
       <c r="M6" t="n">
         <v>0.1201</v>
       </c>
       <c r="N6" t="n">
-        <v>4.5744</v>
+        <v>4.5737</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1016</v>
+        <v>0.1019</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1016</v>
+        <v>0.1019</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.099</v>
+        <v>0.0996</v>
       </c>
       <c r="R6" t="n">
         <v>0.0298</v>
       </c>
       <c r="S6" t="n">
-        <v>6712</v>
+        <v>6713</v>
       </c>
       <c r="T6" t="n">
-        <v>4.6605</v>
+        <v>4.6613</v>
       </c>
       <c r="U6" t="n">
-        <v>25.48</v>
+        <v>25.52</v>
       </c>
       <c r="V6" t="n">
         <v>2.6031</v>
       </c>
       <c r="W6" t="n">
-        <v>2.2607</v>
+        <v>2.2604</v>
       </c>
       <c r="X6" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="Y6" t="n">
         <v>0</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7.917</v>
+        <v>7.919</v>
       </c>
       <c r="B7" t="n">
         <v>73.77056</v>
@@ -1013,64 +1013,64 @@
         <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.6754</v>
+        <v>-0.6742</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.6741</v>
+        <v>-0.673</v>
       </c>
       <c r="G7" t="n">
-        <v>22.291268</v>
+        <v>22.289422</v>
       </c>
       <c r="H7" t="n">
-        <v>22.290335</v>
+        <v>22.288327</v>
       </c>
       <c r="I7" t="n">
-        <v>26.7631</v>
+        <v>26.7595</v>
       </c>
       <c r="J7" t="n">
-        <v>26.7607</v>
+        <v>26.7569</v>
       </c>
       <c r="K7" t="n">
-        <v>371.579</v>
+        <v>371.576</v>
       </c>
       <c r="L7" t="n">
-        <v>362.875</v>
+        <v>362.911</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0885</v>
+        <v>0.0867</v>
       </c>
       <c r="N7" t="n">
-        <v>4.5702</v>
+        <v>4.57</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1025</v>
+        <v>0.1023</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1025</v>
+        <v>0.1023</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1026</v>
+        <v>0.1028</v>
       </c>
       <c r="R7" t="n">
         <v>0.0285</v>
       </c>
       <c r="S7" t="n">
-        <v>6756</v>
+        <v>6757</v>
       </c>
       <c r="T7" t="n">
-        <v>4.6911</v>
+        <v>4.6918</v>
       </c>
       <c r="U7" t="n">
-        <v>24.59</v>
+        <v>24.43</v>
       </c>
       <c r="V7" t="n">
         <v>2.6038</v>
       </c>
       <c r="W7" t="n">
-        <v>2.2611</v>
+        <v>2.2613</v>
       </c>
       <c r="X7" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="Y7" t="n">
         <v>0</v>
@@ -1093,7 +1093,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8.907</v>
+        <v>8.904</v>
       </c>
       <c r="B8" t="n">
         <v>73.77056</v>
@@ -1105,64 +1105,64 @@
         <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.6553</v>
+        <v>-0.6568</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.6637</v>
+        <v>-0.6634</v>
       </c>
       <c r="G8" t="n">
-        <v>22.254781</v>
+        <v>22.255442</v>
       </c>
       <c r="H8" t="n">
-        <v>22.267085</v>
+        <v>22.265609</v>
       </c>
       <c r="I8" t="n">
-        <v>26.697</v>
+        <v>26.6985</v>
       </c>
       <c r="J8" t="n">
-        <v>26.7205</v>
+        <v>26.7179</v>
       </c>
       <c r="K8" t="n">
-        <v>371.795</v>
+        <v>371.85</v>
       </c>
       <c r="L8" t="n">
-        <v>363.339</v>
+        <v>363.443</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1149</v>
+        <v>0.1253</v>
       </c>
       <c r="N8" t="n">
-        <v>4.5713</v>
+        <v>4.5728</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1017</v>
+        <v>0.1018</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1017</v>
+        <v>0.1018</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.1018</v>
+        <v>0.1004</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0296</v>
+        <v>0.03</v>
       </c>
       <c r="S8" t="n">
-        <v>6816</v>
+        <v>6818</v>
       </c>
       <c r="T8" t="n">
-        <v>4.7327</v>
+        <v>4.7338</v>
       </c>
       <c r="U8" t="n">
-        <v>24.1</v>
+        <v>23.94</v>
       </c>
       <c r="V8" t="n">
-        <v>2.605</v>
+        <v>2.6053</v>
       </c>
       <c r="W8" t="n">
-        <v>2.2631</v>
+        <v>2.2636</v>
       </c>
       <c r="X8" t="n">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="Y8" t="n">
         <v>0</v>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9.896</v>
+        <v>9.898</v>
       </c>
       <c r="B9" t="n">
         <v>73.77056</v>
@@ -1197,64 +1197,64 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.6351</v>
+        <v>-0.6357</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.6331</v>
+        <v>-0.635</v>
       </c>
       <c r="G9" t="n">
-        <v>22.251263</v>
+        <v>22.251747</v>
       </c>
       <c r="H9" t="n">
-        <v>22.245263</v>
+        <v>22.251271</v>
       </c>
       <c r="I9" t="n">
-        <v>26.6739</v>
+        <v>26.6741</v>
       </c>
       <c r="J9" t="n">
-        <v>26.6643</v>
+        <v>26.6727</v>
       </c>
       <c r="K9" t="n">
-        <v>371.674</v>
+        <v>371.683</v>
       </c>
       <c r="L9" t="n">
-        <v>363.204</v>
+        <v>363.186</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0808</v>
+        <v>0.0845</v>
       </c>
       <c r="N9" t="n">
-        <v>4.5717</v>
+        <v>4.5722</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1029</v>
+        <v>0.1028</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1029</v>
+        <v>0.1028</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.1013</v>
+        <v>0.101</v>
       </c>
       <c r="R9" t="n">
-        <v>0.0282</v>
+        <v>0.0284</v>
       </c>
       <c r="S9" t="n">
         <v>6863</v>
       </c>
       <c r="T9" t="n">
-        <v>4.7654</v>
+        <v>4.7655</v>
       </c>
       <c r="U9" t="n">
-        <v>23.49</v>
+        <v>23.38</v>
       </c>
       <c r="V9" t="n">
         <v>2.6049</v>
       </c>
       <c r="W9" t="n">
-        <v>2.2631</v>
+        <v>2.263</v>
       </c>
       <c r="X9" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="Y9" t="n">
         <v>0</v>
@@ -1277,7 +1277,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10.886</v>
+        <v>10.887</v>
       </c>
       <c r="B10" t="n">
         <v>73.77056</v>
@@ -1289,64 +1289,64 @@
         <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.6369</v>
+        <v>-0.6358</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.6425</v>
+        <v>-0.6409</v>
       </c>
       <c r="G10" t="n">
-        <v>22.264885</v>
+        <v>22.266608</v>
       </c>
       <c r="H10" t="n">
-        <v>22.283766</v>
+        <v>22.280096</v>
       </c>
       <c r="I10" t="n">
-        <v>26.6929</v>
+        <v>26.6934</v>
       </c>
       <c r="J10" t="n">
-        <v>26.7227</v>
+        <v>26.7157</v>
       </c>
       <c r="K10" t="n">
-        <v>371.496</v>
+        <v>371.431</v>
       </c>
       <c r="L10" t="n">
-        <v>362.619</v>
+        <v>362.543</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1043</v>
+        <v>0.1035</v>
       </c>
       <c r="N10" t="n">
-        <v>4.5753</v>
+        <v>4.5759</v>
       </c>
       <c r="O10" t="n">
-        <v>0.1022</v>
+        <v>0.1024</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1022</v>
+        <v>0.1024</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.0982</v>
+        <v>0.0977</v>
       </c>
       <c r="R10" t="n">
-        <v>0.0292</v>
+        <v>0.0291</v>
       </c>
       <c r="S10" t="n">
-        <v>6911</v>
+        <v>6914</v>
       </c>
       <c r="T10" t="n">
-        <v>4.7986</v>
+        <v>4.8005</v>
       </c>
       <c r="U10" t="n">
-        <v>21.47</v>
+        <v>21.42</v>
       </c>
       <c r="V10" t="n">
-        <v>2.6038</v>
+        <v>2.6035</v>
       </c>
       <c r="W10" t="n">
-        <v>2.2604</v>
+        <v>2.26</v>
       </c>
       <c r="X10" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="Y10" t="n">
         <v>0</v>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11.876</v>
+        <v>11.874</v>
       </c>
       <c r="B11" t="n">
         <v>73.77056</v>
@@ -1381,40 +1381,40 @@
         <v>12</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.6703</v>
+        <v>-0.6704</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.6674</v>
+        <v>-0.6677</v>
       </c>
       <c r="G11" t="n">
-        <v>22.331248</v>
+        <v>22.330448</v>
       </c>
       <c r="H11" t="n">
-        <v>22.326767</v>
+        <v>22.326929</v>
       </c>
       <c r="I11" t="n">
-        <v>26.809</v>
+        <v>26.8086</v>
       </c>
       <c r="J11" t="n">
-        <v>26.8006</v>
+        <v>26.8014</v>
       </c>
       <c r="K11" t="n">
-        <v>371.428</v>
+        <v>371.412</v>
       </c>
       <c r="L11" t="n">
-        <v>362.082</v>
+        <v>362.094</v>
       </c>
       <c r="M11" t="n">
-        <v>0.113</v>
+        <v>0.1116</v>
       </c>
       <c r="N11" t="n">
         <v>4.5759</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1028</v>
+        <v>0.1029</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1028</v>
+        <v>0.1029</v>
       </c>
       <c r="Q11" t="n">
         <v>0.0977</v>
@@ -1423,22 +1423,22 @@
         <v>0.0295</v>
       </c>
       <c r="S11" t="n">
-        <v>6969</v>
+        <v>6970</v>
       </c>
       <c r="T11" t="n">
-        <v>4.839</v>
+        <v>4.8394</v>
       </c>
       <c r="U11" t="n">
-        <v>20.19</v>
+        <v>20.08</v>
       </c>
       <c r="V11" t="n">
-        <v>2.603</v>
+        <v>2.6028</v>
       </c>
       <c r="W11" t="n">
         <v>2.2573</v>
       </c>
       <c r="X11" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="Y11" t="n">
         <v>0</v>
@@ -1461,7 +1461,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12.865</v>
+        <v>12.867</v>
       </c>
       <c r="B12" t="n">
         <v>73.77056</v>
@@ -1473,31 +1473,31 @@
         <v>13</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.6946</v>
+        <v>-0.695</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.6965</v>
+        <v>-0.6971</v>
       </c>
       <c r="G12" t="n">
-        <v>22.389154</v>
+        <v>22.389956</v>
       </c>
       <c r="H12" t="n">
-        <v>22.39706</v>
+        <v>22.39783</v>
       </c>
       <c r="I12" t="n">
-        <v>26.9062</v>
+        <v>26.9088</v>
       </c>
       <c r="J12" t="n">
-        <v>26.9183</v>
+        <v>26.9211</v>
       </c>
       <c r="K12" t="n">
-        <v>371.236</v>
+        <v>371.245</v>
       </c>
       <c r="L12" t="n">
-        <v>362.317</v>
+        <v>362.289</v>
       </c>
       <c r="M12" t="n">
-        <v>0.109</v>
+        <v>0.1098</v>
       </c>
       <c r="N12" t="n">
         <v>4.5743</v>
@@ -1515,22 +1515,22 @@
         <v>0.0294</v>
       </c>
       <c r="S12" t="n">
-        <v>7013</v>
+        <v>7015</v>
       </c>
       <c r="T12" t="n">
-        <v>4.8696</v>
+        <v>4.8706</v>
       </c>
       <c r="U12" t="n">
-        <v>20.07</v>
+        <v>20.1</v>
       </c>
       <c r="V12" t="n">
         <v>2.6017</v>
       </c>
       <c r="W12" t="n">
-        <v>2.2583</v>
+        <v>2.2581</v>
       </c>
       <c r="X12" t="n">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="Y12" t="n">
         <v>0</v>
@@ -1553,7 +1553,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>13.855</v>
+        <v>13.854</v>
       </c>
       <c r="B13" t="n">
         <v>73.77054</v>
@@ -1568,31 +1568,31 @@
         <v>-0.7345</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.7258</v>
+        <v>-0.7275</v>
       </c>
       <c r="G13" t="n">
-        <v>22.512868</v>
+        <v>22.51098</v>
       </c>
       <c r="H13" t="n">
-        <v>22.484303</v>
+        <v>22.488381</v>
       </c>
       <c r="I13" t="n">
-        <v>27.1043</v>
+        <v>27.1037</v>
       </c>
       <c r="J13" t="n">
-        <v>27.0588</v>
+        <v>27.0674</v>
       </c>
       <c r="K13" t="n">
-        <v>371.298</v>
+        <v>371.296</v>
       </c>
       <c r="L13" t="n">
-        <v>363.065</v>
+        <v>363.089</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1351</v>
+        <v>0.1361</v>
       </c>
       <c r="N13" t="n">
-        <v>4.5745</v>
+        <v>4.5749</v>
       </c>
       <c r="O13" t="n">
         <v>0.1042</v>
@@ -1601,28 +1601,28 @@
         <v>0.1042</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.0989</v>
+        <v>0.0986</v>
       </c>
       <c r="R13" t="n">
         <v>0.0304</v>
       </c>
       <c r="S13" t="n">
-        <v>7071</v>
+        <v>7073</v>
       </c>
       <c r="T13" t="n">
-        <v>4.9099</v>
+        <v>4.9109</v>
       </c>
       <c r="U13" t="n">
-        <v>20.95</v>
+        <v>21.05</v>
       </c>
       <c r="V13" t="n">
-        <v>2.6025</v>
+        <v>2.6024</v>
       </c>
       <c r="W13" t="n">
-        <v>2.262</v>
+        <v>2.2621</v>
       </c>
       <c r="X13" t="n">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="Y13" t="n">
         <v>0</v>
@@ -1645,7 +1645,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14.845</v>
+        <v>14.844</v>
       </c>
       <c r="B14" t="n">
         <v>73.77054</v>
@@ -1657,64 +1657,64 @@
         <v>15</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.7446</v>
+        <v>-0.7435</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.7399</v>
+        <v>-0.7395</v>
       </c>
       <c r="G14" t="n">
-        <v>22.540759</v>
+        <v>22.53569</v>
       </c>
       <c r="H14" t="n">
-        <v>22.525742</v>
+        <v>22.523522</v>
       </c>
       <c r="I14" t="n">
-        <v>27.1496</v>
+        <v>27.1436</v>
       </c>
       <c r="J14" t="n">
-        <v>27.1256</v>
+        <v>27.1238</v>
       </c>
       <c r="K14" t="n">
-        <v>371.285</v>
+        <v>371.314</v>
       </c>
       <c r="L14" t="n">
-        <v>362.928</v>
+        <v>362.957</v>
       </c>
       <c r="M14" t="n">
-        <v>0.1331</v>
+        <v>0.1347</v>
       </c>
       <c r="N14" t="n">
         <v>4.576</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1031</v>
+        <v>0.103</v>
       </c>
       <c r="P14" t="n">
-        <v>0.1031</v>
+        <v>0.103</v>
       </c>
       <c r="Q14" t="n">
         <v>0.0976</v>
       </c>
       <c r="R14" t="n">
-        <v>0.0303</v>
+        <v>0.0304</v>
       </c>
       <c r="S14" t="n">
-        <v>7120</v>
+        <v>7121</v>
       </c>
       <c r="T14" t="n">
-        <v>4.9438</v>
+        <v>4.9447</v>
       </c>
       <c r="U14" t="n">
-        <v>18.15</v>
+        <v>18.13</v>
       </c>
       <c r="V14" t="n">
-        <v>2.6022</v>
+        <v>2.6023</v>
       </c>
       <c r="W14" t="n">
-        <v>2.2613</v>
+        <v>2.2614</v>
       </c>
       <c r="X14" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="Y14" t="n">
         <v>0</v>
@@ -1737,7 +1737,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>15.834</v>
+        <v>15.835</v>
       </c>
       <c r="B15" t="n">
         <v>73.77054</v>
@@ -1749,34 +1749,34 @@
         <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.7614</v>
+        <v>-0.7648</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.7644</v>
+        <v>-0.7671</v>
       </c>
       <c r="G15" t="n">
-        <v>22.59067</v>
+        <v>22.598677</v>
       </c>
       <c r="H15" t="n">
-        <v>22.599418</v>
+        <v>22.605335</v>
       </c>
       <c r="I15" t="n">
-        <v>27.23</v>
+        <v>27.2456</v>
       </c>
       <c r="J15" t="n">
-        <v>27.2443</v>
+        <v>27.2566</v>
       </c>
       <c r="K15" t="n">
-        <v>371.369</v>
+        <v>371.378</v>
       </c>
       <c r="L15" t="n">
-        <v>363.143</v>
+        <v>363.303</v>
       </c>
       <c r="M15" t="n">
-        <v>0.135</v>
+        <v>0.1341</v>
       </c>
       <c r="N15" t="n">
-        <v>4.5769</v>
+        <v>4.5776</v>
       </c>
       <c r="O15" t="n">
         <v>0.1053</v>
@@ -1785,28 +1785,28 @@
         <v>0.1053</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.0968</v>
+        <v>0.0962</v>
       </c>
       <c r="R15" t="n">
-        <v>0.0304</v>
+        <v>0.0303</v>
       </c>
       <c r="S15" t="n">
-        <v>7165</v>
+        <v>7166</v>
       </c>
       <c r="T15" t="n">
-        <v>4.975</v>
+        <v>4.9757</v>
       </c>
       <c r="U15" t="n">
-        <v>18.1</v>
+        <v>17.81</v>
       </c>
       <c r="V15" t="n">
-        <v>2.6027</v>
+        <v>2.6028</v>
       </c>
       <c r="W15" t="n">
-        <v>2.2624</v>
+        <v>2.2632</v>
       </c>
       <c r="X15" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -1841,34 +1841,34 @@
         <v>17</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.8141</v>
+        <v>-0.8176</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.806</v>
+        <v>-0.8093</v>
       </c>
       <c r="G16" t="n">
-        <v>22.741076</v>
+        <v>22.750103</v>
       </c>
       <c r="H16" t="n">
-        <v>22.721025</v>
+        <v>22.728812</v>
       </c>
       <c r="I16" t="n">
-        <v>27.4761</v>
+        <v>27.4943</v>
       </c>
       <c r="J16" t="n">
-        <v>27.4421</v>
+        <v>27.4583</v>
       </c>
       <c r="K16" t="n">
-        <v>371.518</v>
+        <v>371.507</v>
       </c>
       <c r="L16" t="n">
-        <v>362.756</v>
+        <v>362.788</v>
       </c>
       <c r="M16" t="n">
-        <v>0.1471</v>
+        <v>0.145</v>
       </c>
       <c r="N16" t="n">
-        <v>4.5811</v>
+        <v>4.5806</v>
       </c>
       <c r="O16" t="n">
         <v>0.1058</v>
@@ -1877,28 +1877,28 @@
         <v>0.1058</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.0931</v>
+        <v>0.0936</v>
       </c>
       <c r="R16" t="n">
-        <v>0.0309</v>
+        <v>0.0308</v>
       </c>
       <c r="S16" t="n">
-        <v>7218</v>
+        <v>7220</v>
       </c>
       <c r="T16" t="n">
-        <v>5.0119</v>
+        <v>5.0133</v>
       </c>
       <c r="U16" t="n">
-        <v>14.75</v>
+        <v>14.56</v>
       </c>
       <c r="V16" t="n">
         <v>2.6039</v>
       </c>
       <c r="W16" t="n">
-        <v>2.2609</v>
+        <v>2.2611</v>
       </c>
       <c r="X16" t="n">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -1921,7 +1921,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>17.813</v>
+        <v>17.812</v>
       </c>
       <c r="B17" t="n">
         <v>73.77054</v>
@@ -1933,64 +1933,64 @@
         <v>18</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.9459</v>
+        <v>-0.9465</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.9386</v>
+        <v>-0.9403</v>
       </c>
       <c r="G17" t="n">
-        <v>23.116592</v>
+        <v>23.111908</v>
       </c>
       <c r="H17" t="n">
-        <v>23.093134</v>
+        <v>23.091979</v>
       </c>
       <c r="I17" t="n">
-        <v>28.0953</v>
+        <v>28.0956</v>
       </c>
       <c r="J17" t="n">
-        <v>28.0572</v>
+        <v>28.0632</v>
       </c>
       <c r="K17" t="n">
-        <v>371.405</v>
+        <v>371.391</v>
       </c>
       <c r="L17" t="n">
-        <v>362.672</v>
+        <v>362.831</v>
       </c>
       <c r="M17" t="n">
-        <v>0.1852</v>
+        <v>0.1879</v>
       </c>
       <c r="N17" t="n">
-        <v>4.5747</v>
+        <v>4.5748</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1087</v>
+        <v>0.1088</v>
       </c>
       <c r="P17" t="n">
-        <v>0.1087</v>
+        <v>0.1088</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.0988</v>
+        <v>0.0987</v>
       </c>
       <c r="R17" t="n">
-        <v>0.0324</v>
+        <v>0.0325</v>
       </c>
       <c r="S17" t="n">
-        <v>7276</v>
+        <v>7277</v>
       </c>
       <c r="T17" t="n">
-        <v>5.0518</v>
+        <v>5.0526</v>
       </c>
       <c r="U17" t="n">
-        <v>12.67</v>
+        <v>12.79</v>
       </c>
       <c r="V17" t="n">
-        <v>2.6048</v>
+        <v>2.6047</v>
       </c>
       <c r="W17" t="n">
-        <v>2.2616</v>
+        <v>2.2624</v>
       </c>
       <c r="X17" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="Y17" t="n">
         <v>0</v>
@@ -2025,64 +2025,64 @@
         <v>19</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.9922</v>
+        <v>-0.9929</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.9908</v>
+        <v>-0.9917</v>
       </c>
       <c r="G18" t="n">
-        <v>23.281673</v>
+        <v>23.279975</v>
       </c>
       <c r="H18" t="n">
-        <v>23.276203</v>
+        <v>23.275164</v>
       </c>
       <c r="I18" t="n">
-        <v>28.3581</v>
+        <v>28.3625</v>
       </c>
       <c r="J18" t="n">
-        <v>28.3495</v>
+        <v>28.355</v>
       </c>
       <c r="K18" t="n">
-        <v>371.948</v>
+        <v>371.956</v>
       </c>
       <c r="L18" t="n">
-        <v>362.685</v>
+        <v>362.692</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2115</v>
+        <v>0.2131</v>
       </c>
       <c r="N18" t="n">
-        <v>4.5684</v>
+        <v>4.5685</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1109</v>
+        <v>0.111</v>
       </c>
       <c r="P18" t="n">
-        <v>0.1109</v>
+        <v>0.111</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.1043</v>
+        <v>0.1042</v>
       </c>
       <c r="R18" t="n">
         <v>0.0335</v>
       </c>
       <c r="S18" t="n">
-        <v>7322</v>
+        <v>7323</v>
       </c>
       <c r="T18" t="n">
-        <v>5.0837</v>
+        <v>5.0844</v>
       </c>
       <c r="U18" t="n">
-        <v>12.34</v>
+        <v>12.33</v>
       </c>
       <c r="V18" t="n">
-        <v>2.6091</v>
+        <v>2.6092</v>
       </c>
       <c r="W18" t="n">
         <v>2.2627</v>
       </c>
       <c r="X18" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="Y18" t="n">
         <v>0</v>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>19.793</v>
+        <v>19.794</v>
       </c>
       <c r="B19" t="n">
         <v>73.77054</v>
@@ -2117,64 +2117,64 @@
         <v>20</v>
       </c>
       <c r="E19" t="n">
-        <v>-1.0151</v>
+        <v>-1.0159</v>
       </c>
       <c r="F19" t="n">
-        <v>-1.0122</v>
+        <v>-1.0126</v>
       </c>
       <c r="G19" t="n">
-        <v>23.324263</v>
+        <v>23.321909</v>
       </c>
       <c r="H19" t="n">
-        <v>23.318122</v>
+        <v>23.315692</v>
       </c>
       <c r="I19" t="n">
-        <v>28.4361</v>
+        <v>28.4389</v>
       </c>
       <c r="J19" t="n">
-        <v>28.4251</v>
+        <v>28.4274</v>
       </c>
       <c r="K19" t="n">
-        <v>373.619</v>
+        <v>373.648</v>
       </c>
       <c r="L19" t="n">
-        <v>364.103</v>
+        <v>364.136</v>
       </c>
       <c r="M19" t="n">
-        <v>0.1994</v>
+        <v>0.199</v>
       </c>
       <c r="N19" t="n">
-        <v>4.5656</v>
+        <v>4.5657</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1122</v>
+        <v>0.1125</v>
       </c>
       <c r="P19" t="n">
-        <v>0.1122</v>
+        <v>0.1125</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.1067</v>
+        <v>0.1066</v>
       </c>
       <c r="R19" t="n">
         <v>0.033</v>
       </c>
       <c r="S19" t="n">
-        <v>7370</v>
+        <v>7371</v>
       </c>
       <c r="T19" t="n">
-        <v>5.1174</v>
+        <v>5.1183</v>
       </c>
       <c r="U19" t="n">
-        <v>11.89</v>
+        <v>11.88</v>
       </c>
       <c r="V19" t="n">
-        <v>2.6181</v>
+        <v>2.6183</v>
       </c>
       <c r="W19" t="n">
-        <v>2.2692</v>
+        <v>2.2694</v>
       </c>
       <c r="X19" t="n">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Y19" t="n">
         <v>0</v>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>20.782</v>
+        <v>20.781</v>
       </c>
       <c r="B20" t="n">
         <v>73.77054</v>
@@ -2209,64 +2209,64 @@
         <v>21</v>
       </c>
       <c r="E20" t="n">
-        <v>-1.1111</v>
+        <v>-1.1123</v>
       </c>
       <c r="F20" t="n">
-        <v>-1.1008</v>
+        <v>-1.1016</v>
       </c>
       <c r="G20" t="n">
-        <v>23.345053</v>
+        <v>23.340953</v>
       </c>
       <c r="H20" t="n">
-        <v>23.344679</v>
+        <v>23.340684</v>
       </c>
       <c r="I20" t="n">
-        <v>28.5546</v>
+        <v>28.5569</v>
       </c>
       <c r="J20" t="n">
-        <v>28.5443</v>
+        <v>28.5462</v>
       </c>
       <c r="K20" t="n">
-        <v>374.695</v>
+        <v>374.728</v>
       </c>
       <c r="L20" t="n">
-        <v>310.23</v>
+        <v>313.559</v>
       </c>
       <c r="M20" t="n">
-        <v>0.1818</v>
+        <v>0.181</v>
       </c>
       <c r="N20" t="n">
-        <v>4.571</v>
+        <v>4.5714</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1131</v>
+        <v>0.1132</v>
       </c>
       <c r="P20" t="n">
-        <v>0.1131</v>
+        <v>0.1132</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.102</v>
+        <v>0.1016</v>
       </c>
       <c r="R20" t="n">
-        <v>0.0323</v>
+        <v>0.0322</v>
       </c>
       <c r="S20" t="n">
-        <v>7427</v>
+        <v>7428</v>
       </c>
       <c r="T20" t="n">
-        <v>5.1569</v>
+        <v>5.1576</v>
       </c>
       <c r="U20" t="n">
-        <v>11.99</v>
+        <v>12.03</v>
       </c>
       <c r="V20" t="n">
-        <v>2.6197</v>
+        <v>2.6199</v>
       </c>
       <c r="W20" t="n">
-        <v>2.0075</v>
+        <v>2.0235</v>
       </c>
       <c r="X20" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -2289,7 +2289,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>21.772</v>
+        <v>21.773</v>
       </c>
       <c r="B21" t="n">
         <v>73.77054</v>
@@ -2301,34 +2301,34 @@
         <v>22</v>
       </c>
       <c r="E21" t="n">
-        <v>-1.1933</v>
+        <v>-1.1946</v>
       </c>
       <c r="F21" t="n">
-        <v>-1.1919</v>
+        <v>-1.1934</v>
       </c>
       <c r="G21" t="n">
-        <v>23.339937</v>
+        <v>23.334368</v>
       </c>
       <c r="H21" t="n">
-        <v>23.338122</v>
+        <v>23.332504</v>
       </c>
       <c r="I21" t="n">
-        <v>28.6257</v>
+        <v>28.6269</v>
       </c>
       <c r="J21" t="n">
-        <v>28.6219</v>
+        <v>28.6234</v>
       </c>
       <c r="K21" t="n">
-        <v>374.14</v>
+        <v>374.117</v>
       </c>
       <c r="L21" t="n">
-        <v>310.164</v>
+        <v>311.659</v>
       </c>
       <c r="M21" t="n">
-        <v>0.306</v>
+        <v>0.31</v>
       </c>
       <c r="N21" t="n">
-        <v>4.5682</v>
+        <v>4.5678</v>
       </c>
       <c r="O21" t="n">
         <v>0.1143</v>
@@ -2337,28 +2337,28 @@
         <v>0.1143</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.1045</v>
+        <v>0.1047</v>
       </c>
       <c r="R21" t="n">
-        <v>0.0372</v>
+        <v>0.0374</v>
       </c>
       <c r="S21" t="n">
-        <v>7475</v>
+        <v>7476</v>
       </c>
       <c r="T21" t="n">
-        <v>5.1903</v>
+        <v>5.1909</v>
       </c>
       <c r="U21" t="n">
-        <v>11.93</v>
+        <v>11.9</v>
       </c>
       <c r="V21" t="n">
-        <v>2.6122</v>
+        <v>2.612</v>
       </c>
       <c r="W21" t="n">
-        <v>2.0036</v>
+        <v>2.0107</v>
       </c>
       <c r="X21" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
@@ -2381,7 +2381,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>22.761</v>
+        <v>22.76</v>
       </c>
       <c r="B22" t="n">
         <v>73.77054</v>
@@ -2393,64 +2393,64 @@
         <v>23</v>
       </c>
       <c r="E22" t="n">
-        <v>-1.2364</v>
+        <v>-1.2382</v>
       </c>
       <c r="F22" t="n">
-        <v>-1.2336</v>
+        <v>-1.2352</v>
       </c>
       <c r="G22" t="n">
-        <v>23.34901</v>
+        <v>23.344196</v>
       </c>
       <c r="H22" t="n">
-        <v>23.346861</v>
+        <v>23.342021</v>
       </c>
       <c r="I22" t="n">
-        <v>28.6786</v>
+        <v>28.6807</v>
       </c>
       <c r="J22" t="n">
-        <v>28.673</v>
+        <v>28.6749</v>
       </c>
       <c r="K22" t="n">
-        <v>371.029</v>
+        <v>370.93</v>
       </c>
       <c r="L22" t="n">
-        <v>304.333</v>
+        <v>305.323</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2916</v>
+        <v>0.2811</v>
       </c>
       <c r="N22" t="n">
-        <v>4.5833</v>
+        <v>4.5844</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1155</v>
+        <v>0.1158</v>
       </c>
       <c r="P22" t="n">
-        <v>0.1155</v>
+        <v>0.1158</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.0913</v>
+        <v>0.0902</v>
       </c>
       <c r="R22" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="S22" t="n">
-        <v>7527</v>
+        <v>7528</v>
       </c>
       <c r="T22" t="n">
-        <v>5.2261</v>
+        <v>5.2274</v>
       </c>
       <c r="U22" t="n">
-        <v>10.89</v>
+        <v>10.85</v>
       </c>
       <c r="V22" t="n">
-        <v>2.5924</v>
+        <v>2.5917</v>
       </c>
       <c r="W22" t="n">
-        <v>1.9743</v>
+        <v>1.979</v>
       </c>
       <c r="X22" t="n">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="Y22" t="n">
         <v>0</v>
@@ -2485,64 +2485,64 @@
         <v>24</v>
       </c>
       <c r="E23" t="n">
-        <v>-1.2639</v>
+        <v>-1.2646</v>
       </c>
       <c r="F23" t="n">
-        <v>-1.2632</v>
+        <v>-1.2638</v>
       </c>
       <c r="G23" t="n">
-        <v>23.366725</v>
+        <v>23.362771</v>
       </c>
       <c r="H23" t="n">
-        <v>23.364742</v>
+        <v>23.360745</v>
       </c>
       <c r="I23" t="n">
-        <v>28.7283</v>
+        <v>28.7296</v>
       </c>
       <c r="J23" t="n">
-        <v>28.7249</v>
+        <v>28.7262</v>
       </c>
       <c r="K23" t="n">
-        <v>367.386</v>
+        <v>367.251</v>
       </c>
       <c r="L23" t="n">
-        <v>294.509</v>
+        <v>300.81</v>
       </c>
       <c r="M23" t="n">
-        <v>0.3403</v>
+        <v>0.3299</v>
       </c>
       <c r="N23" t="n">
-        <v>4.5763</v>
+        <v>4.5725</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1153</v>
+        <v>0.1152</v>
       </c>
       <c r="P23" t="n">
-        <v>0.1153</v>
+        <v>0.1152</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.0974</v>
+        <v>0.1007</v>
       </c>
       <c r="R23" t="n">
-        <v>0.0386</v>
+        <v>0.0382</v>
       </c>
       <c r="S23" t="n">
-        <v>7576</v>
+        <v>7577</v>
       </c>
       <c r="T23" t="n">
-        <v>5.2602</v>
+        <v>5.2608</v>
       </c>
       <c r="U23" t="n">
-        <v>10.38</v>
+        <v>10.37</v>
       </c>
       <c r="V23" t="n">
-        <v>2.5706</v>
+        <v>2.5698</v>
       </c>
       <c r="W23" t="n">
-        <v>1.9264</v>
+        <v>1.9565</v>
       </c>
       <c r="X23" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -2577,64 +2577,64 @@
         <v>25</v>
       </c>
       <c r="E24" t="n">
-        <v>-1.2867</v>
+        <v>-1.2872</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.2849</v>
+        <v>-1.2854</v>
       </c>
       <c r="G24" t="n">
-        <v>23.387257</v>
+        <v>23.384169</v>
       </c>
       <c r="H24" t="n">
-        <v>23.384681</v>
+        <v>23.381701</v>
       </c>
       <c r="I24" t="n">
-        <v>28.7774</v>
+        <v>28.7787</v>
       </c>
       <c r="J24" t="n">
-        <v>28.7721</v>
+        <v>28.7736</v>
       </c>
       <c r="K24" t="n">
-        <v>361.779</v>
+        <v>361.544</v>
       </c>
       <c r="L24" t="n">
-        <v>355.069</v>
+        <v>353.999</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2435</v>
+        <v>0.2448</v>
       </c>
       <c r="N24" t="n">
-        <v>4.5866</v>
+        <v>4.5874</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1164</v>
+        <v>0.1165</v>
       </c>
       <c r="P24" t="n">
-        <v>0.1164</v>
+        <v>0.1165</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.0884</v>
+        <v>0.0877</v>
       </c>
       <c r="R24" t="n">
-        <v>0.0347</v>
+        <v>0.0348</v>
       </c>
       <c r="S24" t="n">
-        <v>7629</v>
+        <v>7631</v>
       </c>
       <c r="T24" t="n">
-        <v>5.2969</v>
+        <v>5.2985</v>
       </c>
       <c r="U24" t="n">
-        <v>9.78</v>
+        <v>9.75</v>
       </c>
       <c r="V24" t="n">
-        <v>2.5379</v>
+        <v>2.5366</v>
       </c>
       <c r="W24" t="n">
-        <v>2.2151</v>
+        <v>2.21</v>
       </c>
       <c r="X24" t="n">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="Y24" t="n">
         <v>0</v>
@@ -2657,7 +2657,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>25.73</v>
+        <v>25.729</v>
       </c>
       <c r="B25" t="n">
         <v>73.77054</v>
@@ -2669,64 +2669,64 @@
         <v>26</v>
       </c>
       <c r="E25" t="n">
-        <v>-1.3181</v>
+        <v>-1.3193</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.3157</v>
+        <v>-1.3169</v>
       </c>
       <c r="G25" t="n">
-        <v>23.400464</v>
+        <v>23.39734</v>
       </c>
       <c r="H25" t="n">
-        <v>23.398754</v>
+        <v>23.395526</v>
       </c>
       <c r="I25" t="n">
-        <v>28.8249</v>
+        <v>28.8264</v>
       </c>
       <c r="J25" t="n">
-        <v>28.8203</v>
+        <v>28.8216</v>
       </c>
       <c r="K25" t="n">
-        <v>356.258</v>
+        <v>356.194</v>
       </c>
       <c r="L25" t="n">
-        <v>351.804</v>
+        <v>351.758</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2259</v>
+        <v>0.2238</v>
       </c>
       <c r="N25" t="n">
-        <v>4.5911</v>
+        <v>4.5913</v>
       </c>
       <c r="O25" t="n">
-        <v>0.1174</v>
+        <v>0.1172</v>
       </c>
       <c r="P25" t="n">
-        <v>0.1174</v>
+        <v>0.1172</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.0844</v>
+        <v>0.0842</v>
       </c>
       <c r="R25" t="n">
-        <v>0.0341</v>
+        <v>0.034</v>
       </c>
       <c r="S25" t="n">
-        <v>7685</v>
+        <v>7686</v>
       </c>
       <c r="T25" t="n">
-        <v>5.336</v>
+        <v>5.3367</v>
       </c>
       <c r="U25" t="n">
-        <v>5.79</v>
+        <v>5.29</v>
       </c>
       <c r="V25" t="n">
-        <v>2.5053</v>
+        <v>2.5049</v>
       </c>
       <c r="W25" t="n">
-        <v>2.1984</v>
+        <v>2.1981</v>
       </c>
       <c r="X25" t="n">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="Y25" t="n">
         <v>0</v>
@@ -2749,7 +2749,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>26.719</v>
+        <v>26.72</v>
       </c>
       <c r="B26" t="n">
         <v>73.77054</v>
@@ -2761,64 +2761,64 @@
         <v>27</v>
       </c>
       <c r="E26" t="n">
-        <v>-1.3465</v>
+        <v>-1.3471</v>
       </c>
       <c r="F26" t="n">
-        <v>-1.3442</v>
+        <v>-1.3448</v>
       </c>
       <c r="G26" t="n">
-        <v>23.417148</v>
+        <v>23.41481</v>
       </c>
       <c r="H26" t="n">
-        <v>23.414451</v>
+        <v>23.41211</v>
       </c>
       <c r="I26" t="n">
-        <v>28.8744</v>
+        <v>28.876</v>
       </c>
       <c r="J26" t="n">
-        <v>28.8685</v>
+        <v>28.8702</v>
       </c>
       <c r="K26" t="n">
-        <v>352.062</v>
+        <v>351.852</v>
       </c>
       <c r="L26" t="n">
-        <v>346.751</v>
+        <v>346.625</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1921</v>
+        <v>0.1907</v>
       </c>
       <c r="N26" t="n">
-        <v>4.6006</v>
+        <v>4.6005</v>
       </c>
       <c r="O26" t="n">
-        <v>0.1148</v>
+        <v>0.1152</v>
       </c>
       <c r="P26" t="n">
-        <v>0.1148</v>
+        <v>0.1152</v>
       </c>
       <c r="Q26" t="n">
         <v>0.0762</v>
       </c>
       <c r="R26" t="n">
-        <v>0.0327</v>
+        <v>0.0326</v>
       </c>
       <c r="S26" t="n">
-        <v>7732</v>
+        <v>7734</v>
       </c>
       <c r="T26" t="n">
-        <v>5.3688</v>
+        <v>5.3699</v>
       </c>
       <c r="U26" t="n">
-        <v>0.12</v>
+        <v>0.26</v>
       </c>
       <c r="V26" t="n">
-        <v>2.4804</v>
+        <v>2.4792</v>
       </c>
       <c r="W26" t="n">
-        <v>2.1732</v>
+        <v>2.1726</v>
       </c>
       <c r="X26" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="Y26" t="n">
         <v>0</v>
@@ -2853,31 +2853,31 @@
         <v>28</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.3687</v>
+        <v>-1.369</v>
       </c>
       <c r="F27" t="n">
-        <v>-1.3666</v>
+        <v>-1.367</v>
       </c>
       <c r="G27" t="n">
-        <v>23.44393</v>
+        <v>23.442094</v>
       </c>
       <c r="H27" t="n">
-        <v>23.440629</v>
+        <v>23.438701</v>
       </c>
       <c r="I27" t="n">
-        <v>28.9315</v>
+        <v>28.9331</v>
       </c>
       <c r="J27" t="n">
-        <v>28.925</v>
+        <v>28.9266</v>
       </c>
       <c r="K27" t="n">
-        <v>345.688</v>
+        <v>345.528</v>
       </c>
       <c r="L27" t="n">
-        <v>342.203</v>
+        <v>342.095</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1701</v>
+        <v>0.167</v>
       </c>
       <c r="N27" t="n">
         <v>4.6041</v>
@@ -2892,25 +2892,25 @@
         <v>0.0731</v>
       </c>
       <c r="R27" t="n">
-        <v>0.0318</v>
+        <v>0.0317</v>
       </c>
       <c r="S27" t="n">
-        <v>7784</v>
+        <v>7785</v>
       </c>
       <c r="T27" t="n">
-        <v>5.4047</v>
+        <v>5.4056</v>
       </c>
       <c r="U27" t="n">
         <v>0.01</v>
       </c>
       <c r="V27" t="n">
-        <v>2.4437</v>
+        <v>2.4428</v>
       </c>
       <c r="W27" t="n">
-        <v>2.1509</v>
+        <v>2.1504</v>
       </c>
       <c r="X27" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="Y27" t="n">
         <v>0</v>
@@ -2933,7 +2933,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>28.698</v>
+        <v>28.7</v>
       </c>
       <c r="B28" t="n">
         <v>73.77052</v>
@@ -2945,34 +2945,34 @@
         <v>29</v>
       </c>
       <c r="E28" t="n">
-        <v>-1.3808</v>
+        <v>-1.3813</v>
       </c>
       <c r="F28" t="n">
-        <v>-1.3793</v>
+        <v>-1.3798</v>
       </c>
       <c r="G28" t="n">
-        <v>23.477784</v>
+        <v>23.475696</v>
       </c>
       <c r="H28" t="n">
-        <v>23.47459</v>
+        <v>23.472615</v>
       </c>
       <c r="I28" t="n">
-        <v>28.9885</v>
+        <v>28.9893</v>
       </c>
       <c r="J28" t="n">
-        <v>28.9827</v>
+        <v>28.9837</v>
       </c>
       <c r="K28" t="n">
-        <v>339.136</v>
+        <v>338.892</v>
       </c>
       <c r="L28" t="n">
-        <v>336.09</v>
+        <v>335.767</v>
       </c>
       <c r="M28" t="n">
-        <v>0.1262</v>
+        <v>0.1245</v>
       </c>
       <c r="N28" t="n">
-        <v>4.6099</v>
+        <v>4.6103</v>
       </c>
       <c r="O28" t="n">
         <v>0.116</v>
@@ -2981,28 +2981,28 @@
         <v>0.116</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.0681</v>
+        <v>0.0677</v>
       </c>
       <c r="R28" t="n">
         <v>0.03</v>
       </c>
       <c r="S28" t="n">
-        <v>7836</v>
+        <v>7838</v>
       </c>
       <c r="T28" t="n">
-        <v>5.441</v>
+        <v>5.4426</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
       </c>
       <c r="V28" t="n">
-        <v>2.4066</v>
+        <v>2.4052</v>
       </c>
       <c r="W28" t="n">
-        <v>2.1216</v>
+        <v>2.1201</v>
       </c>
       <c r="X28" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="Y28" t="n">
         <v>0</v>
@@ -3037,64 +3037,64 @@
         <v>30</v>
       </c>
       <c r="E29" t="n">
-        <v>-1.3943</v>
+        <v>-1.3947</v>
       </c>
       <c r="F29" t="n">
-        <v>-1.3916</v>
+        <v>-1.3918</v>
       </c>
       <c r="G29" t="n">
-        <v>23.500881</v>
+        <v>23.499832</v>
       </c>
       <c r="H29" t="n">
-        <v>23.496793</v>
+        <v>23.495594</v>
       </c>
       <c r="I29" t="n">
-        <v>29.0322</v>
+        <v>29.0336</v>
       </c>
       <c r="J29" t="n">
-        <v>29.0241</v>
+        <v>29.025</v>
       </c>
       <c r="K29" t="n">
-        <v>332.839</v>
+        <v>332.585</v>
       </c>
       <c r="L29" t="n">
-        <v>328.641</v>
+        <v>328.318</v>
       </c>
       <c r="M29" t="n">
-        <v>0.1382</v>
+        <v>0.1401</v>
       </c>
       <c r="N29" t="n">
-        <v>4.6143</v>
+        <v>4.6147</v>
       </c>
       <c r="O29" t="n">
-        <v>0.1157</v>
+        <v>0.1158</v>
       </c>
       <c r="P29" t="n">
-        <v>0.1157</v>
+        <v>0.1158</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.0643</v>
+        <v>0.0639</v>
       </c>
       <c r="R29" t="n">
-        <v>0.0305</v>
+        <v>0.0306</v>
       </c>
       <c r="S29" t="n">
-        <v>7914</v>
+        <v>7920</v>
       </c>
       <c r="T29" t="n">
-        <v>5.4953</v>
+        <v>5.499</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>2.3707</v>
+        <v>2.3692</v>
       </c>
       <c r="W29" t="n">
-        <v>2.0858</v>
+        <v>2.0843</v>
       </c>
       <c r="X29" t="n">
-        <v>21</v>
+        <v>103</v>
       </c>
       <c r="Y29" t="n">
         <v>0</v>
@@ -3129,64 +3129,64 @@
         <v>31</v>
       </c>
       <c r="E30" t="n">
-        <v>-1.4092</v>
+        <v>-1.4096</v>
       </c>
       <c r="F30" t="n">
-        <v>-1.4081</v>
+        <v>-1.4084</v>
       </c>
       <c r="G30" t="n">
-        <v>23.536207</v>
+        <v>23.538475</v>
       </c>
       <c r="H30" t="n">
-        <v>23.532131</v>
+        <v>23.533678</v>
       </c>
       <c r="I30" t="n">
-        <v>29.094</v>
+        <v>29.0993</v>
       </c>
       <c r="J30" t="n">
-        <v>29.0874</v>
+        <v>29.0916</v>
       </c>
       <c r="K30" t="n">
-        <v>328.286</v>
+        <v>328.159</v>
       </c>
       <c r="L30" t="n">
-        <v>323.318</v>
+        <v>323.191</v>
       </c>
       <c r="M30" t="n">
-        <v>0.118</v>
+        <v>0.1196</v>
       </c>
       <c r="N30" t="n">
-        <v>4.6194</v>
+        <v>4.6184</v>
       </c>
       <c r="O30" t="n">
-        <v>0.1161</v>
+        <v>0.1159</v>
       </c>
       <c r="P30" t="n">
-        <v>0.1161</v>
+        <v>0.1159</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.0598</v>
+        <v>0.0607</v>
       </c>
       <c r="R30" t="n">
-        <v>0.0297</v>
+        <v>0.0298</v>
       </c>
       <c r="S30" t="n">
-        <v>8013</v>
+        <v>8016</v>
       </c>
       <c r="T30" t="n">
-        <v>5.5636</v>
+        <v>5.5658</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>2.3448</v>
+        <v>2.3441</v>
       </c>
       <c r="W30" t="n">
-        <v>2.0602</v>
+        <v>2.0597</v>
       </c>
       <c r="X30" t="n">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="Y30" t="n">
         <v>0</v>
@@ -3221,34 +3221,34 @@
         <v>32</v>
       </c>
       <c r="E31" t="n">
-        <v>-1.4176</v>
+        <v>-1.4181</v>
       </c>
       <c r="F31" t="n">
-        <v>-1.4162</v>
+        <v>-1.4166</v>
       </c>
       <c r="G31" t="n">
-        <v>23.588386</v>
+        <v>23.589825</v>
       </c>
       <c r="H31" t="n">
-        <v>23.581966</v>
+        <v>23.582851</v>
       </c>
       <c r="I31" t="n">
-        <v>29.1724</v>
+        <v>29.176</v>
       </c>
       <c r="J31" t="n">
-        <v>29.1624</v>
+        <v>29.1651</v>
       </c>
       <c r="K31" t="n">
-        <v>320.279</v>
+        <v>319.876</v>
       </c>
       <c r="L31" t="n">
-        <v>317.239</v>
+        <v>316.932</v>
       </c>
       <c r="M31" t="n">
-        <v>0.1533</v>
+        <v>0.1521</v>
       </c>
       <c r="N31" t="n">
-        <v>4.6122</v>
+        <v>4.6115</v>
       </c>
       <c r="O31" t="n">
         <v>0.1177</v>
@@ -3257,28 +3257,28 @@
         <v>0.1177</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.066</v>
+        <v>0.0666</v>
       </c>
       <c r="R31" t="n">
         <v>0.0311</v>
       </c>
       <c r="S31" t="n">
-        <v>8111</v>
+        <v>8116</v>
       </c>
       <c r="T31" t="n">
-        <v>5.6321</v>
+        <v>5.6352</v>
       </c>
       <c r="U31" t="n">
         <v>0.09</v>
       </c>
       <c r="V31" t="n">
-        <v>2.3</v>
+        <v>2.2978</v>
       </c>
       <c r="W31" t="n">
-        <v>2.0316</v>
+        <v>2.0301</v>
       </c>
       <c r="X31" t="n">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="Y31" t="n">
         <v>0</v>
@@ -3319,28 +3319,28 @@
         <v>-1.4178</v>
       </c>
       <c r="G32" t="n">
-        <v>23.719906</v>
+        <v>23.72514</v>
       </c>
       <c r="H32" t="n">
-        <v>23.709625</v>
+        <v>23.71401</v>
       </c>
       <c r="I32" t="n">
-        <v>29.3508</v>
+        <v>29.3586</v>
       </c>
       <c r="J32" t="n">
-        <v>29.3364</v>
+        <v>29.3431</v>
       </c>
       <c r="K32" t="n">
-        <v>309.676</v>
+        <v>309.271</v>
       </c>
       <c r="L32" t="n">
-        <v>307.437</v>
+        <v>307.061</v>
       </c>
       <c r="M32" t="n">
-        <v>0.3483</v>
+        <v>0.357</v>
       </c>
       <c r="N32" t="n">
-        <v>4.6011</v>
+        <v>4.6003</v>
       </c>
       <c r="O32" t="n">
         <v>0.1172</v>
@@ -3349,28 +3349,28 @@
         <v>0.1172</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.0756</v>
+        <v>0.0763</v>
       </c>
       <c r="R32" t="n">
-        <v>0.039</v>
+        <v>0.0393</v>
       </c>
       <c r="S32" t="n">
-        <v>8205</v>
+        <v>8209</v>
       </c>
       <c r="T32" t="n">
-        <v>5.6973</v>
+        <v>5.6999</v>
       </c>
       <c r="U32" t="n">
         <v>0.05</v>
       </c>
       <c r="V32" t="n">
-        <v>2.2424</v>
+        <v>2.2402</v>
       </c>
       <c r="W32" t="n">
-        <v>1.9866</v>
+        <v>1.9848</v>
       </c>
       <c r="X32" t="n">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="Y32" t="n">
         <v>0</v>
@@ -3405,64 +3405,64 @@
         <v>34</v>
       </c>
       <c r="E33" t="n">
-        <v>-1.4471</v>
+        <v>-1.4482</v>
       </c>
       <c r="F33" t="n">
-        <v>-1.4457</v>
+        <v>-1.4469</v>
       </c>
       <c r="G33" t="n">
-        <v>23.906389</v>
+        <v>23.909574</v>
       </c>
       <c r="H33" t="n">
-        <v>23.901803</v>
+        <v>23.904838</v>
       </c>
       <c r="I33" t="n">
-        <v>29.6318</v>
+        <v>29.6385</v>
       </c>
       <c r="J33" t="n">
-        <v>29.6243</v>
+        <v>29.6307</v>
       </c>
       <c r="K33" t="n">
-        <v>302.447</v>
+        <v>301.75</v>
       </c>
       <c r="L33" t="n">
-        <v>299.614</v>
+        <v>299.21</v>
       </c>
       <c r="M33" t="n">
-        <v>0.5446</v>
+        <v>0.5414</v>
       </c>
       <c r="N33" t="n">
-        <v>4.5338</v>
+        <v>4.5281</v>
       </c>
       <c r="O33" t="n">
-        <v>0.1193</v>
+        <v>0.1194</v>
       </c>
       <c r="P33" t="n">
-        <v>0.1193</v>
+        <v>0.1194</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.1349</v>
+        <v>0.1399</v>
       </c>
       <c r="R33" t="n">
-        <v>0.0468</v>
+        <v>0.0467</v>
       </c>
       <c r="S33" t="n">
-        <v>8300</v>
+        <v>8305</v>
       </c>
       <c r="T33" t="n">
-        <v>5.7629</v>
+        <v>5.7666</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>2.2036</v>
+        <v>2.1997</v>
       </c>
       <c r="W33" t="n">
-        <v>1.9511</v>
+        <v>1.9491</v>
       </c>
       <c r="X33" t="n">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="Y33" t="n">
         <v>0</v>
@@ -3497,34 +3497,34 @@
         <v>35</v>
       </c>
       <c r="E34" t="n">
-        <v>-1.4594</v>
+        <v>-1.4596</v>
       </c>
       <c r="F34" t="n">
-        <v>-1.459</v>
+        <v>-1.4591</v>
       </c>
       <c r="G34" t="n">
-        <v>23.955108</v>
+        <v>23.955117</v>
       </c>
       <c r="H34" t="n">
-        <v>23.953341</v>
+        <v>23.953088</v>
       </c>
       <c r="I34" t="n">
-        <v>29.7098</v>
+        <v>29.7109</v>
       </c>
       <c r="J34" t="n">
-        <v>29.707</v>
+        <v>29.7077</v>
       </c>
       <c r="K34" t="n">
-        <v>285.934</v>
+        <v>285.414</v>
       </c>
       <c r="L34" t="n">
-        <v>285.44</v>
+        <v>284.806</v>
       </c>
       <c r="M34" t="n">
-        <v>0.5313</v>
+        <v>0.5411</v>
       </c>
       <c r="N34" t="n">
-        <v>4.3988</v>
+        <v>4.3928</v>
       </c>
       <c r="O34" t="n">
         <v>0.1203</v>
@@ -3533,28 +3533,28 @@
         <v>0.1203</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.256</v>
+        <v>0.2614</v>
       </c>
       <c r="R34" t="n">
-        <v>0.0463</v>
+        <v>0.0466</v>
       </c>
       <c r="S34" t="n">
-        <v>8399</v>
+        <v>8402</v>
       </c>
       <c r="T34" t="n">
-        <v>5.8318</v>
+        <v>5.8342</v>
       </c>
       <c r="U34" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="V34" t="n">
-        <v>2.1103</v>
+        <v>2.1074</v>
       </c>
       <c r="W34" t="n">
-        <v>1.8834</v>
+        <v>1.8804</v>
       </c>
       <c r="X34" t="n">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="Y34" t="n">
         <v>0</v>
@@ -3592,31 +3592,31 @@
         <v>-1.4625</v>
       </c>
       <c r="F35" t="n">
-        <v>-1.4622</v>
+        <v>-1.4621</v>
       </c>
       <c r="G35" t="n">
-        <v>23.967503</v>
+        <v>23.966839</v>
       </c>
       <c r="H35" t="n">
-        <v>23.966022</v>
+        <v>23.965388</v>
       </c>
       <c r="I35" t="n">
-        <v>29.7291</v>
+        <v>29.7288</v>
       </c>
       <c r="J35" t="n">
-        <v>29.7268</v>
+        <v>29.7265</v>
       </c>
       <c r="K35" t="n">
-        <v>274.842</v>
+        <v>274.624</v>
       </c>
       <c r="L35" t="n">
-        <v>273.353</v>
+        <v>273.043</v>
       </c>
       <c r="M35" t="n">
-        <v>0.5497</v>
+        <v>0.5473</v>
       </c>
       <c r="N35" t="n">
-        <v>4.1899</v>
+        <v>4.181</v>
       </c>
       <c r="O35" t="n">
         <v>0.1202</v>
@@ -3625,28 +3625,28 @@
         <v>0.1202</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.451</v>
+        <v>0.4596</v>
       </c>
       <c r="R35" t="n">
-        <v>0.047</v>
+        <v>0.0469</v>
       </c>
       <c r="S35" t="n">
-        <v>8492</v>
+        <v>8496</v>
       </c>
       <c r="T35" t="n">
-        <v>5.8967</v>
+        <v>5.8996</v>
       </c>
       <c r="U35" t="n">
         <v>0.06</v>
       </c>
       <c r="V35" t="n">
-        <v>2.0475</v>
+        <v>2.0462</v>
       </c>
       <c r="W35" t="n">
-        <v>1.8256</v>
+        <v>1.8241</v>
       </c>
       <c r="X35" t="n">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="Y35" t="n">
         <v>0</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>36.615</v>
+        <v>36.614</v>
       </c>
       <c r="B36" t="n">
         <v>73.77052</v>
@@ -3687,58 +3687,58 @@
         <v>-1.4623</v>
       </c>
       <c r="G36" t="n">
-        <v>23.966911</v>
+        <v>23.966675</v>
       </c>
       <c r="H36" t="n">
-        <v>23.965787</v>
+        <v>23.965595</v>
       </c>
       <c r="I36" t="n">
         <v>29.7279</v>
       </c>
       <c r="J36" t="n">
-        <v>29.726</v>
+        <v>29.7261</v>
       </c>
       <c r="K36" t="n">
-        <v>271.375</v>
+        <v>271.196</v>
       </c>
       <c r="L36" t="n">
-        <v>268.438</v>
+        <v>268.178</v>
       </c>
       <c r="M36" t="n">
-        <v>0.5804</v>
+        <v>0.5812</v>
       </c>
       <c r="N36" t="n">
-        <v>4.0912</v>
+        <v>4.088</v>
       </c>
       <c r="O36" t="n">
-        <v>0.1208</v>
+        <v>0.1209</v>
       </c>
       <c r="P36" t="n">
-        <v>0.1208</v>
+        <v>0.1209</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.5461</v>
+        <v>0.5492</v>
       </c>
       <c r="R36" t="n">
         <v>0.0482</v>
       </c>
       <c r="S36" t="n">
-        <v>8589</v>
+        <v>8593</v>
       </c>
       <c r="T36" t="n">
-        <v>5.9638</v>
+        <v>5.9664</v>
       </c>
       <c r="U36" t="n">
         <v>0.04</v>
       </c>
       <c r="V36" t="n">
-        <v>2.0276</v>
+        <v>2.0266</v>
       </c>
       <c r="W36" t="n">
-        <v>1.8019</v>
+        <v>1.8006</v>
       </c>
       <c r="X36" t="n">
-        <v>19</v>
+        <v>91</v>
       </c>
       <c r="Y36" t="n">
         <v>0</v>
@@ -3761,7 +3761,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>37.604</v>
+        <v>37.608</v>
       </c>
       <c r="B37" t="n">
         <v>73.77052</v>
@@ -3773,64 +3773,64 @@
         <v>38</v>
       </c>
       <c r="E37" t="n">
-        <v>-1.4608</v>
+        <v>-1.4614</v>
       </c>
       <c r="F37" t="n">
-        <v>-1.46</v>
+        <v>-1.4599</v>
       </c>
       <c r="G37" t="n">
-        <v>23.959467</v>
+        <v>23.961487</v>
       </c>
       <c r="H37" t="n">
-        <v>23.958536</v>
+        <v>23.957778</v>
       </c>
       <c r="I37" t="n">
-        <v>29.7154</v>
+        <v>29.7187</v>
       </c>
       <c r="J37" t="n">
-        <v>29.7133</v>
+        <v>29.7122</v>
       </c>
       <c r="K37" t="n">
-        <v>269.202</v>
+        <v>269.006</v>
       </c>
       <c r="L37" t="n">
-        <v>265.36</v>
+        <v>264.869</v>
       </c>
       <c r="M37" t="n">
-        <v>0.6159</v>
+        <v>0.6667</v>
       </c>
       <c r="N37" t="n">
-        <v>3.8416</v>
+        <v>3.8044</v>
       </c>
       <c r="O37" t="n">
-        <v>0.1205</v>
+        <v>0.1209</v>
       </c>
       <c r="P37" t="n">
-        <v>0.1205</v>
+        <v>0.1209</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.7969</v>
+        <v>0.8346</v>
       </c>
       <c r="R37" t="n">
-        <v>0.0496</v>
+        <v>0.0517</v>
       </c>
       <c r="S37" t="n">
-        <v>9310</v>
+        <v>9322</v>
       </c>
       <c r="T37" t="n">
-        <v>6.4645</v>
+        <v>6.473</v>
       </c>
       <c r="U37" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="V37" t="n">
-        <v>2.015</v>
+        <v>2.0139</v>
       </c>
       <c r="W37" t="n">
-        <v>1.787</v>
+        <v>1.7846</v>
       </c>
       <c r="X37" t="n">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="Y37" t="n">
         <v>0</v>

</xml_diff>